<commit_message>
Updated flow factor plot
</commit_message>
<xml_diff>
--- a/data/workshop/flow-factors.xlsx
+++ b/data/workshop/flow-factors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://birminghamcitycouncil-my.sharepoint.com/personal/david_ellis_birmingham_gov_uk/Documents/Documents/Documents/MPH/Measles Modelling/Measles-System-Dynamics-BSol/data/workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_F25DC773A252ABDACC1048C4315C7F365BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96AFE052-23A1-48E9-9EC3-A7F8189481DB}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="11_F25DC773A252ABDACC1048C4315C7F365BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBC4AF30-EE74-4853-9D7E-759D828B8E43}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,12 +48,6 @@
     <t>Community Norms</t>
   </si>
   <si>
-    <t>System factors</t>
-  </si>
-  <si>
-    <t>Social factors</t>
-  </si>
-  <si>
     <t>Family Influence/Experience</t>
   </si>
   <si>
@@ -85,6 +79,12 @@
   </si>
   <si>
     <t>Information</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>Social</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C2">
         <v>7</v>
@@ -445,7 +445,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -456,7 +456,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -467,7 +467,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -475,10 +475,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -486,10 +486,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -508,10 +508,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -519,10 +519,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C10">
         <v>6</v>
@@ -530,10 +530,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -541,10 +541,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -552,10 +552,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
         <v>16</v>
-      </c>
-      <c r="B13" t="s">
-        <v>18</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -563,10 +563,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C14">
         <v>1</v>

</xml_diff>